<commit_message>
Add new Excel file 'perfil_subtipos.xlsx' with initial content
</commit_message>
<xml_diff>
--- a/resumo_pvalores.xlsx
+++ b/resumo_pvalores.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I40"/>
+  <dimension ref="A1:I43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1976,6 +1976,123 @@
         </is>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Tamanho da lesão × Ulceração</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>414</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Mann-Whitney</t>
+        </is>
+      </c>
+      <c r="F41" t="n">
+        <v>13479.5</v>
+      </c>
+      <c r="G41" t="n">
+        <v>0</v>
+      </c>
+      <c r="H41" t="n">
+        <v>0.313</v>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>F2</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Tamanho da lesão × Margens comprometidas</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>415</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Mann-Whitney</t>
+        </is>
+      </c>
+      <c r="F42" t="n">
+        <v>7979</v>
+      </c>
+      <c r="G42" t="n">
+        <v>0.0706</v>
+      </c>
+      <c r="H42" t="n">
+        <v>0.155</v>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>F3</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Tamanho da lesão × Invasão perineural</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>414</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Mann-Whitney</t>
+        </is>
+      </c>
+      <c r="F43" t="n">
+        <v>2411.5</v>
+      </c>
+      <c r="G43" t="n">
+        <v>0.0033</v>
+      </c>
+      <c r="H43" t="n">
+        <v>0.388</v>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>